<commit_message>
Fixed CUL+DRY cows scenario and name change RET_COWS -> CUL_COWS
</commit_message>
<xml_diff>
--- a/scenarios/DRY_COWS.xlsx
+++ b/scenarios/DRY_COWS.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="36">
   <si>
     <t>parameter</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>all other feeds reduced proportionally</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
 </sst>
 </file>
@@ -134,7 +137,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,6 +168,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -186,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -194,9 +211,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,14 +555,14 @@
       <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="11">
         <f>K2</f>
         <v>9452.1428570000007</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="11">
         <v>10025.4</v>
       </c>
-      <c r="K2" s="4">
+      <c r="K2" s="12">
         <v>9452.1428570000007</v>
       </c>
       <c r="L2" t="s">
@@ -561,14 +582,14 @@
       <c r="G3" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="11">
         <f>K3</f>
         <v>8631.0214290000004</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="11">
         <v>9367.2000000000007</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="12">
         <v>8631.0214290000004</v>
       </c>
       <c r="L3" t="s">
@@ -595,7 +616,7 @@
       <c r="J5">
         <v>13.2</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="13">
         <v>14</v>
       </c>
       <c r="L5" t="s">
@@ -622,7 +643,7 @@
       <c r="J6">
         <v>12.9</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="13">
         <v>14</v>
       </c>
       <c r="L6" t="s">
@@ -649,7 +670,7 @@
       <c r="J8">
         <v>37.1</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="9">
         <v>35.4</v>
       </c>
       <c r="L8" t="s">
@@ -676,7 +697,7 @@
       <c r="J9">
         <v>36.1</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="9">
         <v>33.5</v>
       </c>
       <c r="L9" t="s">
@@ -698,15 +719,18 @@
       <c r="G11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H11" s="7">
-        <f>J11</f>
+      <c r="H11" s="4">
+        <f>K11</f>
         <v>651.52821361702138</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="4">
         <v>651.52821361702138</v>
       </c>
-      <c r="K11" s="4"/>
+      <c r="K11" s="10">
+        <f>J11</f>
+        <v>651.52821361702138</v>
+      </c>
       <c r="L11" t="s">
         <v>26</v>
       </c>
@@ -764,7 +788,7 @@
       <c r="J14" s="1">
         <v>6.6079520088655128</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="9">
         <v>16.5</v>
       </c>
     </row>
@@ -781,7 +805,7 @@
       <c r="G15" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="7">
         <f>(1 / (100 - J$14)) * (1 - K$14/100) * 100</f>
         <v>0.89408040401819311</v>
       </c>
@@ -818,7 +842,7 @@
       <c r="J16" s="1">
         <v>6.4615074492035101</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="9">
         <v>16.5</v>
       </c>
     </row>
@@ -841,7 +865,7 @@
       <c r="G17" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="7">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
         <v>0.89268062508763379</v>
       </c>
@@ -899,8 +923,8 @@
       <c r="J1" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="9" t="s">
-        <v>18</v>
+      <c r="K1" s="8" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -932,7 +956,7 @@
       <c r="J2" s="2">
         <v>20</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="9">
         <v>50</v>
       </c>
       <c r="L2" t="s">

</xml_diff>